<commit_message>
working on PICCOmela and imports+ revisions of ClimOO-SDC2
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations/ClimOO Imports.xlsx
+++ b/ClimOO material/materials for implementations/ClimOO Imports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ECE0C8A-92A7-7B44-8445-185DF8C68F92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{849C6A8B-86DF-1941-8642-0584146848F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16460" activeTab="1" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
+    <workbookView xWindow="33000" yWindow="520" windowWidth="28800" windowHeight="16440" xr2:uid="{BC4974B6-08E4-914F-B6A6-1E86DBDCF25D}"/>
   </bookViews>
   <sheets>
     <sheet name="PlasticO imports" sheetId="3" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="367">
   <si>
     <t>Agri-Food Experiment Ontology</t>
   </si>
@@ -1135,6 +1135,12 @@
   </si>
   <si>
     <t xml:space="preserve">https://oborel.github.io/ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes </t>
+  </si>
+  <si>
+    <t>Mapped to BFO</t>
   </si>
 </sst>
 </file>
@@ -1307,7 +1313,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1360,7 +1366,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Collegamento ipertestuale" xfId="1" builtinId="8"/>
@@ -1765,7 +1770,7 @@
         <v>359</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>65</v>
+        <v>365</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
@@ -1891,7 +1896,7 @@
         <v>241</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>68</v>
+        <v>366</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -1988,10 +1993,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D1D5A97-5CAC-5842-B2F3-5274D7CBD229}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="10.83203125" style="32"/>
+    <col min="4" max="4" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
@@ -2033,7 +2038,7 @@
         <v>359</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>65</v>
+        <v>365</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="26" customFormat="1" ht="15" x14ac:dyDescent="0.2">
@@ -2106,6 +2111,20 @@
       </c>
       <c r="D8" s="3" t="s">
         <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>243</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>242</v>
+      </c>
+      <c r="C9" s="16" t="s">
+        <v>241</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>366</v>
       </c>
     </row>
   </sheetData>
@@ -2117,6 +2136,7 @@
     <hyperlink ref="C6" r:id="rId5" xr:uid="{6FF9D3D0-63B1-434F-A4BF-A7D96AAEBD50}"/>
     <hyperlink ref="C8" r:id="rId6" xr:uid="{B2E5C9E1-6D7E-6546-8243-BCE0B3C2C6CD}"/>
     <hyperlink ref="C7" r:id="rId7" xr:uid="{E0037802-D06E-EC48-82DA-3BDF4AD4F7FC}"/>
+    <hyperlink ref="C9" r:id="rId8" xr:uid="{A1311309-7DFD-7B44-9B2F-C93B1FD256E3}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>